<commit_message>
Updating the model for Necaluxan
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Solar.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Solar.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,7 +394,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46283</v>
+        <v>46285</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -402,7 +402,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46283.01041666666</v>
+        <v>46285.01041666666</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -410,7 +410,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46283.02083333334</v>
+        <v>46285.02083333334</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -418,7 +418,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46283.03125</v>
+        <v>46285.03125</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -426,7 +426,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46283.04166666666</v>
+        <v>46285.04166666666</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -434,7 +434,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46283.05208333334</v>
+        <v>46285.05208333334</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -442,7 +442,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46283.0625</v>
+        <v>46285.0625</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,7 +450,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46283.07291666666</v>
+        <v>46285.07291666666</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -458,7 +458,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46283.08333333334</v>
+        <v>46285.08333333334</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -466,7 +466,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46283.09375</v>
+        <v>46285.09375</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -474,7 +474,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46283.10416666666</v>
+        <v>46285.10416666666</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46283.11458333334</v>
+        <v>46285.11458333334</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -490,7 +490,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46283.125</v>
+        <v>46285.125</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -498,7 +498,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46283.13541666666</v>
+        <v>46285.13541666666</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46283.14583333334</v>
+        <v>46285.14583333334</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -514,7 +514,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46283.15625</v>
+        <v>46285.15625</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46283.16666666666</v>
+        <v>46285.16666666666</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -530,7 +530,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46283.17708333334</v>
+        <v>46285.17708333334</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46283.1875</v>
+        <v>46285.1875</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46283.19791666666</v>
+        <v>46285.19791666666</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46283.20833333334</v>
+        <v>46285.20833333334</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -562,7 +562,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46283.21875</v>
+        <v>46285.21875</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46283.22916666666</v>
+        <v>46285.22916666666</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46283.23958333334</v>
+        <v>46285.23958333334</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -586,130 +586,114 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46283.25</v>
+        <v>46285.25</v>
       </c>
       <c r="B26">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46283.26041666666</v>
+        <v>46285.26041666666</v>
       </c>
       <c r="B27">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46283.27083333334</v>
+        <v>46285.27083333334</v>
       </c>
       <c r="B28">
-        <v>132</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46283.28125</v>
+        <v>46285.28125</v>
       </c>
       <c r="B29">
-        <v>273</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46283.29166666666</v>
+        <v>46285.29166666666</v>
       </c>
       <c r="B30">
-        <v>448</v>
+        <v>339</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46283.30208333334</v>
+        <v>46285.30208333334</v>
       </c>
       <c r="B31">
-        <v>622</v>
+        <v>529</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46283.3125</v>
+        <v>46285.3125</v>
       </c>
       <c r="B32">
-        <v>622</v>
+        <v>729</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46283.32291666666</v>
+        <v>46285.32291666666</v>
       </c>
       <c r="B33">
-        <v>998</v>
+        <v>938</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46283.33333333334</v>
+        <v>46285.33333333334</v>
       </c>
       <c r="B34">
-        <v>998</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46283.34375</v>
+        <v>46285.34375</v>
       </c>
       <c r="B35">
-        <v>998</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46283.35416666666</v>
+        <v>46285.35416666666</v>
       </c>
       <c r="B36">
-        <v>1554</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46283.36458333334</v>
+        <v>46285.36458333334</v>
       </c>
       <c r="B37">
-        <v>1704</v>
+        <v>1614</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46283.375</v>
+        <v>46285.375</v>
       </c>
       <c r="B38">
-        <v>1813</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46283.38541666666</v>
+        <v>46285.38541666666</v>
       </c>
       <c r="B39">
-        <v>1948</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="2">
-        <v>46283.39583333334</v>
-      </c>
-      <c r="B40">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" s="2">
-        <v>46283.40625</v>
-      </c>
-      <c r="B41">
-        <v>2062</v>
+        <v>1912</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the model for Ferma Frumusica
</commit_message>
<xml_diff>
--- a/data_fetching/Entsoe/Actual_Production_Solar.xlsx
+++ b/data_fetching/Entsoe/Actual_Production_Solar.xlsx
@@ -381,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -394,7 +394,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -402,7 +402,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2">
-        <v>46307.01041666666</v>
+        <v>46308.01041666666</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -410,7 +410,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2">
-        <v>46307.02083333334</v>
+        <v>46308.02083333334</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -418,7 +418,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2">
-        <v>46307.03125</v>
+        <v>46308.03125</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -426,7 +426,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2">
-        <v>46307.04166666666</v>
+        <v>46308.04166666666</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -434,7 +434,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2">
-        <v>46307.05208333334</v>
+        <v>46308.05208333334</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -442,7 +442,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2">
-        <v>46307.0625</v>
+        <v>46308.0625</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -450,7 +450,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2">
-        <v>46307.07291666666</v>
+        <v>46308.07291666666</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -458,7 +458,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2">
-        <v>46307.08333333334</v>
+        <v>46308.08333333334</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -466,7 +466,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2">
-        <v>46307.09375</v>
+        <v>46308.09375</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -474,7 +474,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2">
-        <v>46307.10416666666</v>
+        <v>46308.10416666666</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2">
-        <v>46307.11458333334</v>
+        <v>46308.11458333334</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -490,7 +490,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2">
-        <v>46307.125</v>
+        <v>46308.125</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -498,7 +498,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2">
-        <v>46307.13541666666</v>
+        <v>46308.13541666666</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -506,7 +506,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2">
-        <v>46307.14583333334</v>
+        <v>46308.14583333334</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -514,7 +514,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2">
-        <v>46307.15625</v>
+        <v>46308.15625</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -522,7 +522,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2">
-        <v>46307.16666666666</v>
+        <v>46308.16666666666</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -530,7 +530,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2">
-        <v>46307.17708333334</v>
+        <v>46308.17708333334</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2">
-        <v>46307.1875</v>
+        <v>46308.1875</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2">
-        <v>46307.19791666666</v>
+        <v>46308.19791666666</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="2">
-        <v>46307.20833333334</v>
+        <v>46308.20833333334</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -562,7 +562,7 @@
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="2">
-        <v>46307.21875</v>
+        <v>46308.21875</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="2">
-        <v>46307.22916666666</v>
+        <v>46308.22916666666</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="2">
-        <v>46307.23958333334</v>
+        <v>46308.23958333334</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -586,7 +586,7 @@
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="2">
-        <v>46307.25</v>
+        <v>46308.25</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -594,7 +594,7 @@
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="2">
-        <v>46307.26041666666</v>
+        <v>46308.26041666666</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="28" spans="1:2">
       <c r="A28" s="2">
-        <v>46307.27083333334</v>
+        <v>46308.27083333334</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -610,7 +610,7 @@
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="2">
-        <v>46307.28125</v>
+        <v>46308.28125</v>
       </c>
       <c r="B29">
         <v>1</v>
@@ -618,90 +618,218 @@
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="2">
-        <v>46307.29166666666</v>
+        <v>46308.29166666666</v>
       </c>
       <c r="B30">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="2">
-        <v>46307.30208333334</v>
+        <v>46308.30208333334</v>
       </c>
       <c r="B31">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="2">
-        <v>46307.3125</v>
+        <v>46308.3125</v>
       </c>
       <c r="B32">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="2">
-        <v>46307.32291666666</v>
+        <v>46308.32291666666</v>
       </c>
       <c r="B33">
-        <v>180</v>
+        <v>207</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="2">
-        <v>46307.33333333334</v>
+        <v>46308.33333333334</v>
       </c>
       <c r="B34">
-        <v>252</v>
+        <v>305</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="2">
-        <v>46307.34375</v>
+        <v>46308.34375</v>
       </c>
       <c r="B35">
-        <v>315</v>
+        <v>405</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="2">
-        <v>46307.35416666666</v>
+        <v>46308.35416666666</v>
       </c>
       <c r="B36">
-        <v>398</v>
+        <v>487</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="2">
-        <v>46307.36458333334</v>
+        <v>46308.36458333334</v>
       </c>
       <c r="B37">
-        <v>461</v>
+        <v>583</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2">
-        <v>46307.375</v>
+        <v>46308.375</v>
       </c>
       <c r="B38">
-        <v>547</v>
+        <v>689</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="2">
-        <v>46307.38541666666</v>
+        <v>46308.38541666666</v>
       </c>
       <c r="B39">
-        <v>594</v>
+        <v>772</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2">
-        <v>46307.39583333334</v>
+        <v>46308.39583333334</v>
       </c>
       <c r="B40">
-        <v>684</v>
+        <v>842</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="2">
+        <v>46308.40625</v>
+      </c>
+      <c r="B41">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="2">
+        <v>46308.41666666666</v>
+      </c>
+      <c r="B42">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="2">
+        <v>46308.42708333334</v>
+      </c>
+      <c r="B43">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="2">
+        <v>46308.4375</v>
+      </c>
+      <c r="B44">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="2">
+        <v>46308.44791666666</v>
+      </c>
+      <c r="B45">
+        <v>1199</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="2">
+        <v>46308.45833333334</v>
+      </c>
+      <c r="B46">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="2">
+        <v>46308.46875</v>
+      </c>
+      <c r="B47">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="2">
+        <v>46308.47916666666</v>
+      </c>
+      <c r="B48">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="2">
+        <v>46308.48958333334</v>
+      </c>
+      <c r="B49">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="2">
+        <v>46308.5</v>
+      </c>
+      <c r="B50">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="2">
+        <v>46308.51041666666</v>
+      </c>
+      <c r="B51">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="2">
+        <v>46308.52083333334</v>
+      </c>
+      <c r="B52">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="2">
+        <v>46308.53125</v>
+      </c>
+      <c r="B53">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="2">
+        <v>46308.54166666666</v>
+      </c>
+      <c r="B54">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="2">
+        <v>46308.55208333334</v>
+      </c>
+      <c r="B55">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="2">
+        <v>46308.5625</v>
+      </c>
+      <c r="B56">
+        <v>1183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>